<commit_message>
Extractos: Impuesto de Sellos, Suscripción Periódico Acción e intereses por saldo deudor como gastos
- Nuevas categorías de gasto: "Impuesto de Sellos" y "Suscripción Periódico Acción"
  (esta última se considera gasto bancario a pedido de administración)
- "Intereses por Saldo Deudor" (Credicoop) se suma a la categoría Intereses
- Extracto ficticio de Credicoop y tests actualizados con los tres conceptos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/extracto-credicoop.xlsx
+++ b/e2e/fixtures/extracto-credicoop.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>1054395.45</v>
+        <v>1021986.03</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -453,7 +453,7 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1069075.5</v>
+        <v>1036666.08</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -473,7 +473,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1073450.5</v>
+        <v>1041041.08</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -481,19 +481,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>20/07/2026</v>
+        <v>28/07/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>Servicio acreditaciones automaticas SERV ACRED AUTOMATIC-0001</v>
+        <v>Intereses por Saldo Deudor</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>9074.42</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1138450.5</v>
+        <v>1106041.08</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -504,16 +504,16 @@
         <v>20/07/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>Comision por Transferencia B. INTERNET COM. USO-0001</v>
+        <v>Impuesto de Sellos - Chaco</v>
       </c>
       <c r="C6">
-        <v>500</v>
+        <v>23335</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>1138480.5</v>
+        <v>1115115.5</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -521,19 +521,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>15/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>Suscripcion al Periodico Accion</v>
+        <v>Servicio acreditaciones automaticas SERV ACRED AUTOMATIC-0001</v>
       </c>
       <c r="C7">
-        <v>2000</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>1138980.5</v>
+        <v>1138450.5</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -541,19 +541,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>15/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>Debito/Credito Aut - Segurcoop Comercio SEGUR.SOCIO-123</v>
+        <v>Comision por Transferencia B. INTERNET COM. USO-0001</v>
       </c>
       <c r="C8">
-        <v>5000</v>
+        <v>500</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>1140980.5</v>
+        <v>1138480.5</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -561,19 +561,19 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>12/07/2026</v>
+        <v>15/07/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>Impuesto Ley 25.413 Ali Gral s/Debitos</v>
+        <v>Suscripcion al Periodico Accion</v>
       </c>
       <c r="C9">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>1145980.5</v>
+        <v>1138980.5</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -581,19 +581,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>12/07/2026</v>
+        <v>15/07/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>Transf.Inmediata e/Ctas.Igual Tit.O/Bco 0000001-VAR-TITULAR FICTICIA</v>
+        <v>Debito/Credito Aut - Segurcoop Comercio SEGUR.SOCIO-123</v>
       </c>
       <c r="C10">
-        <v>300000</v>
+        <v>5000</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1147780.5</v>
+        <v>1140980.5</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -601,19 +601,19 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>09/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>Transf. Inmediata e/Ctas. Dist. Titular 30733333339-FAC-OBRA SOCIAL TRES CBU Origen: 0110599520000055518882</v>
+        <v>Impuesto Ley 25.413 Ali Gral s/Debitos</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="D11">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>1447780.5</v>
+        <v>1145980.5</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -621,19 +621,19 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>05/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>Impuesto Ley 25.413 Ali Gral s/Creditos</v>
+        <v>Transf.Inmediata e/Ctas.Igual Tit.O/Bco 0000001-VAR-TITULAR FICTICIA</v>
       </c>
       <c r="C12">
-        <v>720</v>
+        <v>300000</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>1367780.5</v>
+        <v>1147780.5</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -641,19 +641,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>05/07/2026</v>
+        <v>09/07/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>Transf. Interbanking - Distinto Titular Ord.:30722222225-OBRA SOCIAL FICTICIA</v>
+        <v>Transf. Inmediata e/Ctas. Dist. Titular 30733333339-FAC-OBRA SOCIAL TRES CBU Origen: 0110599520000055518882</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="E13">
-        <v>1368500.5</v>
+        <v>1447780.5</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -661,19 +661,19 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>02/07/2026</v>
+        <v>05/07/2026</v>
       </c>
       <c r="B14" t="str">
         <v>Impuesto Ley 25.413 Ali Gral s/Creditos</v>
       </c>
       <c r="C14">
-        <v>1500</v>
+        <v>720</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1248500.5</v>
+        <v>1367780.5</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -681,27 +681,67 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>05/07/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Transf. Interbanking - Distinto Titular Ord.:30722222225-OBRA SOCIAL FICTICIA</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>120000</v>
+      </c>
+      <c r="E15">
+        <v>1368500.5</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>02/07/2026</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
+        <v>Impuesto Ley 25.413 Ali Gral s/Creditos</v>
+      </c>
+      <c r="C16">
+        <v>1500</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>1248500.5</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>02/07/2026</v>
+      </c>
+      <c r="B17" t="str">
         <v>Transf. Recibida o/Banco-Dist. Titular PROVEED-30711111111-CUENTAFICTICIA</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
         <v>250000.5</v>
       </c>
-      <c r="E15">
+      <c r="E17">
         <v>1250000.5</v>
       </c>
-      <c r="F15" t="str">
+      <c r="F17" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>